<commit_message>
docs: accept menu inventory baseline and study menu IA options
- Record owner acceptance D-135..D-141: v1.0 is the approved baseline,
  ID freeze does not freeze names, prices, categories or availability,
  Arabic names reviewed later in category groups, pending items marked
  ACTIVE - DATA INCOMPLETE
- Mark the v1.0 workbook as approved baseline (product data unchanged)
- Add 22: menu information architecture study with options A/B/C,
  a nine-criteria comparison, answers to the 15 questions and a
  recommendation (C); no UI or components yet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013mm8KaYh9F3CgRAWgw9FwG
</commit_message>
<xml_diff>
--- a/docs/phase-01-discovery/menu/SHELTER-MENU-INVENTORY-v1.0.xlsx
+++ b/docs/phase-01-discovery/menu/SHELTER-MENU-INVENTORY-v1.0.xlsx
@@ -503,7 +503,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SHELTER COFFEE — MENU INVENTORY v1.0 (FROZEN IDs)</t>
+          <t>SHELTER COFFEE — MENU INVENTORY v1.0 — APPROVED BASELINE (D-135)</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>D-091 — اعتماد دفعة واحدة ممكن</t>
+          <t>D-137: مراجعة لاحقة بمجموعات حسب الفئة؛ المشكوك فيه فقط منفردًا · لا تمنع Menu IA</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>المصدر "آيس شيكن سولتد" · مقترح: "آيس شيكن سولتد كراميل"</t>
+          <t>PENDING OWNER APPROVAL (D-138) · المصدر "آيس شيكن سولتد"</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1119,6 +1119,53 @@
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>D-134</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>CHG-00005</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>MV-2026-10-01</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>BASELINE_APPROVED</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>MENU INVENTORY v1.0</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED BASELINE</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>D-135</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1311,7 @@
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>v1.0 (FROZEN IDs)</t>
+          <t>v1.0 — APPROVED BASELINE</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1386,7 +1433,19 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>4 (PND-001 → PND-004)</t>
+          <t>4 (PND-001 → PND-004) — ACTIVE — DATA INCOMPLETE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Baseline status</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED BASELINE (D-135) — تجميد المعرّفات لا يجمّد الاسم أو السعر أو الفئة أو التوفر أو الصورة أو الوصف أو الحالة (D-136)</t>
         </is>
       </c>
     </row>
@@ -68660,7 +68719,7 @@
     <row r="1" ht="44" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>152 صنفًا + 9 فئات: أسماء عربية من ملفك لم تُعتمد بعد كأسماء عرض (D-091). يمكن اعتمادها دفعة واحدة كما هي.</t>
+          <t>152 صنفًا + 9 فئات: SOURCE-PROVIDED — PENDING OWNER REVIEW (D-091، D-137). المراجعة لاحقًا بمجموعات حسب الفئة.</t>
         </is>
       </c>
     </row>
@@ -73243,7 +73302,7 @@
     <row r="1" ht="44" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>ليست ضمن المعرّفات المجمّدة. تأخذ PRD-00193 وما بعده عند وصول الاسم الرسمي والسعر والفئة.</t>
+          <t>ليست ضمن المعرّفات المجمّدة. لا سعر ولا فئة ولا معرّف نهائي من عندنا (D-140). تأخذ PRD-00193 وما بعده عند وصول بياناتها منك.</t>
         </is>
       </c>
     </row>
@@ -73322,7 +73381,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>ACTIVE PRODUCT — MISSING CURRENT MENU DATA</t>
+          <t>ACTIVE — DATA INCOMPLETE</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -73384,7 +73443,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>ACTIVE PRODUCT — MISSING CURRENT MENU DATA</t>
+          <t>ACTIVE — DATA INCOMPLETE</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -73446,7 +73505,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>ACTIVE PRODUCT — MISSING CURRENT MENU DATA</t>
+          <t>ACTIVE — DATA INCOMPLETE</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -73508,7 +73567,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>ACTIVE PRODUCT — MISSING CURRENT MENU DATA</t>
+          <t>ACTIVE — DATA INCOMPLETE</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -73570,7 +73629,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>STATUS UNKNOWN — OWNER VERIFICATION REQUIRED</t>
+          <t>OWNER VERIFICATION REQUIRED</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -73632,7 +73691,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>STATUS UNKNOWN — OWNER VERIFICATION REQUIRED</t>
+          <t>OWNER VERIFICATION REQUIRED</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">

</xml_diff>